<commit_message>
Revisión: VPH sin genotipificar, medicación de la colposcopia en el D1, voz sin nombre opcional, planillas con precios nuevos (v1.19.1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MG6VeavRZnDbjYZyzDjvL
</commit_message>
<xml_diff>
--- a/docs/negocio/SIVEC-metrica-Bolivia.xlsx
+++ b/docs/negocio/SIVEC-metrica-Bolivia.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Fases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Supostos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Departamentos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Municípios" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Equipe" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Ferramentas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supostos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Departamentos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Municípios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipe" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ferramentas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,10 +22,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="$#,##0;($#,##0);-"/>
-    <numFmt numFmtId="165" formatCode="0.0%;(0.0%);-"/>
-    <numFmt numFmtId="166" formatCode="#,##0;(#,##0);-"/>
-    <numFmt numFmtId="167" formatCode="&quot;Bs&quot; #,##0;(&quot;Bs&quot; #,##0);-"/>
+    <numFmt numFmtId="164" formatCode="#,##0;(#,##0);-"/>
+    <numFmt numFmtId="165" formatCode="$#,##0;($#,##0);-"/>
+    <numFmt numFmtId="166" formatCode="&quot;Bs&quot; #,##0;(&quot;Bs&quot; #,##0);-"/>
+    <numFmt numFmtId="167" formatCode="0.0%;(0.0%);-"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -137,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,33 +145,50 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -606,7 +623,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -640,18 +656,18 @@
           <t>Redes</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="6">
+      <c r="B5" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="33">
         <f>'Municípios'!D5</f>
         <v/>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="33">
         <f>Departamentos!C5</f>
         <v/>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="33">
         <f>Departamentos!C14</f>
         <v/>
       </c>
@@ -662,18 +678,18 @@
           <t>Centros 1º nível</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="32" t="n">
         <v>9</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="33">
         <f>'Municípios'!E5</f>
         <v/>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="33">
         <f>Departamentos!D5</f>
         <v/>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="33">
         <f>Departamentos!D14</f>
         <v/>
       </c>
@@ -684,18 +700,18 @@
           <t>Hospitais 2º nível</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="6">
+      <c r="B7" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="33">
         <f>'Municípios'!F5</f>
         <v/>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="33">
         <f>Departamentos!E5</f>
         <v/>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="33">
         <f>Departamentos!E14</f>
         <v/>
       </c>
@@ -706,18 +722,18 @@
           <t>3º nível + labs + oncológico</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="6">
+      <c r="B8" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="33">
         <f>'Municípios'!G5</f>
         <v/>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="33">
         <f>Departamentos!F5</f>
         <v/>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="33">
         <f>Departamentos!F14</f>
         <v/>
       </c>
@@ -728,19 +744,19 @@
           <t>Receita bruta mensal (US$)</t>
         </is>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="34">
         <f>B5*Supostos!$B$8+B6*Supostos!$B$5+B7*Supostos!$B$6+B8*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="34">
         <f>C5*Supostos!$B$8+C6*Supostos!$B$5+C7*Supostos!$B$6+C8*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="34">
         <f>D5*Supostos!$B$8+D6*Supostos!$B$5+D7*Supostos!$B$6+D8*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="34">
         <f>E5*Supostos!$B$8+E6*Supostos!$B$5+E7*Supostos!$B$6+E8*Supostos!$B$7</f>
         <v/>
       </c>
@@ -751,19 +767,19 @@
           <t>Receita bruta anual (US$)</t>
         </is>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="34">
         <f>B9*12</f>
         <v/>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="34">
         <f>C9*12</f>
         <v/>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="34">
         <f>D9*12</f>
         <v/>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="34">
         <f>E9*12</f>
         <v/>
       </c>
@@ -774,19 +790,19 @@
           <t>Receita bruta anual (Bs)</t>
         </is>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="35">
         <f>B10*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="35">
         <f>C10*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="35">
         <f>D10*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="35">
         <f>E10*Supostos!$B$9</f>
         <v/>
       </c>
@@ -797,19 +813,19 @@
           <t>(−) Impostos sobre faturamento (US$/ano)</t>
         </is>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="34">
         <f>-B10*Supostos!$B$10</f>
         <v/>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="34">
         <f>-C10*Supostos!$B$10</f>
         <v/>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="34">
         <f>-D10*Supostos!$B$10</f>
         <v/>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="34">
         <f>-E10*Supostos!$B$10</f>
         <v/>
       </c>
@@ -820,19 +836,19 @@
           <t>Receita líquida anual (US$)</t>
         </is>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="34">
         <f>B10+B12</f>
         <v/>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="34">
         <f>C10+C12</f>
         <v/>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="34">
         <f>D10+D12</f>
         <v/>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="34">
         <f>E10+E12</f>
         <v/>
       </c>
@@ -843,19 +859,19 @@
           <t>(−) Equipe (US$/ano)</t>
         </is>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="36">
         <f>-Equipe!I22/Supostos!$B$9*12</f>
         <v/>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="36">
         <f>-Equipe!J22/Supostos!$B$9*12</f>
         <v/>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="36">
         <f>-Equipe!K22/Supostos!$B$9*12</f>
         <v/>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="36">
         <f>-Equipe!L22/Supostos!$B$9*12</f>
         <v/>
       </c>
@@ -866,19 +882,19 @@
           <t>(−) Ferramentas e operação (US$/ano)</t>
         </is>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="36">
         <f>-Ferramentas!E22*12</f>
         <v/>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="36">
         <f>-Ferramentas!F22*12</f>
         <v/>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="36">
         <f>-Ferramentas!G22*12</f>
         <v/>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="36">
         <f>-Ferramentas!H22*12</f>
         <v/>
       </c>
@@ -889,19 +905,19 @@
           <t>Resultado antes do IUE (US$/ano)</t>
         </is>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="34">
         <f>B13+B14+B15</f>
         <v/>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="34">
         <f>C13+C14+C15</f>
         <v/>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="34">
         <f>D13+D14+D15</f>
         <v/>
       </c>
-      <c r="E16" s="8">
+      <c r="E16" s="34">
         <f>E13+E14+E15</f>
         <v/>
       </c>
@@ -912,19 +928,19 @@
           <t>(−) IUE (US$/ano)</t>
         </is>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="34">
         <f>-MAX(0,B16)*Supostos!$B$11</f>
         <v/>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="34">
         <f>-MAX(0,C16)*Supostos!$B$11</f>
         <v/>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="34">
         <f>-MAX(0,D16)*Supostos!$B$11</f>
         <v/>
       </c>
-      <c r="E17" s="8">
+      <c r="E17" s="34">
         <f>-MAX(0,E16)*Supostos!$B$11</f>
         <v/>
       </c>
@@ -935,19 +951,19 @@
           <t>Lucro líquido anual (US$)</t>
         </is>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="37">
         <f>B16+B17</f>
         <v/>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="37">
         <f>C16+C17</f>
         <v/>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="37">
         <f>D16+D17</f>
         <v/>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="37">
         <f>E16+E17</f>
         <v/>
       </c>
@@ -958,19 +974,19 @@
           <t>Lucro líquido anual (Bs)</t>
         </is>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="38">
         <f>B18*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="38">
         <f>C18*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="D19" s="13">
+      <c r="D19" s="38">
         <f>D18*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="E19" s="13">
+      <c r="E19" s="38">
         <f>E18*Supostos!$B$9</f>
         <v/>
       </c>
@@ -981,19 +997,19 @@
           <t>Margem líquida (% da receita bruta)</t>
         </is>
       </c>
-      <c r="B20" s="14">
+      <c r="B20" s="39">
         <f>IFERROR(B18/B10,0)</f>
         <v/>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="39">
         <f>IFERROR(C18/C10,0)</f>
         <v/>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="39">
         <f>IFERROR(D18/D10,0)</f>
         <v/>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="39">
         <f>IFERROR(E18/E10,0)</f>
         <v/>
       </c>
@@ -1004,19 +1020,19 @@
           <t>Pessoas na equipe</t>
         </is>
       </c>
-      <c r="B21" s="6">
+      <c r="B21" s="33">
         <f>Equipe!E22</f>
         <v/>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="33">
         <f>Equipe!F22</f>
         <v/>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="33">
         <f>Equipe!G22</f>
         <v/>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="33">
         <f>Equipe!H22</f>
         <v/>
       </c>
@@ -1027,24 +1043,23 @@
           <t>Estabelecimentos atendidos</t>
         </is>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="40">
         <f>B6+B7+B8</f>
         <v/>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="40">
         <f>C6+C7+C8</f>
         <v/>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="40">
         <f>D6+D7+D8</f>
         <v/>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="40">
         <f>E6+E7+E8</f>
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
@@ -1113,7 +1128,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1137,8 +1151,8 @@
           <t>Preço mensal · centro de 1º nível (US$)</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
-        <v>100</v>
+      <c r="B5" s="41" t="n">
+        <v>120</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
@@ -1152,8 +1166,8 @@
           <t>Preço mensal · hospital de 2º nível (US$)</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
-        <v>250</v>
+      <c r="B6" s="41" t="n">
+        <v>275</v>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
@@ -1167,8 +1181,8 @@
           <t>Preço mensal · 3º nível, laboratório e oncológico (US$)</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
-        <v>501</v>
+      <c r="B7" s="41" t="n">
+        <v>521</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
@@ -1182,8 +1196,8 @@
           <t>Preço mensal · rede de saúde (tablero do gestor + mapa) (US$)</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n">
-        <v>300</v>
+      <c r="B8" s="42" t="n">
+        <v>250</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -1212,7 +1226,7 @@
           <t>Impostos sobre o faturamento (IVA 13% + IT 3%)</t>
         </is>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="43" t="n">
         <v>0.16</v>
       </c>
       <c r="C10" s="19" t="inlineStr">
@@ -1227,7 +1241,7 @@
           <t>Imposto sobre o lucro (IUE)</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="43" t="n">
         <v>0.25</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -1242,7 +1256,7 @@
           <t>Encargos sociais sobre salário (patronais + aguinaldo + indenização)</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="44" t="n">
         <v>0.33</v>
       </c>
       <c r="C12" s="19" t="inlineStr">
@@ -1251,8 +1265,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
@@ -1329,7 +1341,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1393,34 +1404,34 @@
           <t>Santa Cruz</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="32" t="n">
         <v>3122605</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="32" t="n">
         <v>19</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="45" t="n">
         <v>796</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="45" t="n">
         <v>52</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="45" t="n">
         <v>13</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="34">
         <f>C5*Supostos!$B$8+D5*Supostos!$B$5+E5*Supostos!$B$6+F5*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="34">
         <f>G5*12</f>
         <v/>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="35">
         <f>G5*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="35">
         <f>H5*Supostos!$B$9</f>
         <v/>
       </c>
@@ -1436,34 +1447,34 @@
           <t>La Paz</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="32" t="n">
         <v>3030917</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="45" t="n">
         <v>864</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="45" t="n">
         <v>57</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="45" t="n">
         <v>13</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="34">
         <f>C6*Supostos!$B$8+D6*Supostos!$B$5+E6*Supostos!$B$6+F6*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="34">
         <f>G6*12</f>
         <v/>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="35">
         <f>G6*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="35">
         <f>H6*Supostos!$B$9</f>
         <v/>
       </c>
@@ -1479,34 +1490,34 @@
           <t>Cochabamba</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="45" t="n">
         <v>2005000</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="32" t="n">
         <v>485</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="32" t="n">
         <v>56</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="45" t="n">
         <v>7</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="34">
         <f>C7*Supostos!$B$8+D7*Supostos!$B$5+E7*Supostos!$B$6+F7*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="34">
         <f>G7*12</f>
         <v/>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="35">
         <f>G7*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="35">
         <f>H7*Supostos!$B$9</f>
         <v/>
       </c>
@@ -1522,34 +1533,34 @@
           <t>Potosí</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="45" t="n">
         <v>856000</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="32" t="n">
         <v>11</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="45" t="n">
         <v>314</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="45" t="n">
         <v>21</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="34">
         <f>C8*Supostos!$B$8+D8*Supostos!$B$5+E8*Supostos!$B$6+F8*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="34">
         <f>G8*12</f>
         <v/>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="35">
         <f>G8*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J8" s="9">
+      <c r="J8" s="35">
         <f>H8*Supostos!$B$9</f>
         <v/>
       </c>
@@ -1565,34 +1576,34 @@
           <t>Chuquisaca</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="45" t="n">
         <v>600000</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="32" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="45" t="n">
         <v>208</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="45" t="n">
         <v>14</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="34">
         <f>C9*Supostos!$B$8+D9*Supostos!$B$5+E9*Supostos!$B$6+F9*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="34">
         <f>G9*12</f>
         <v/>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="35">
         <f>G9*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="35">
         <f>H9*Supostos!$B$9</f>
         <v/>
       </c>
@@ -1608,34 +1619,34 @@
           <t>Oruro</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
+      <c r="B10" s="45" t="n">
         <v>570000</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="45" t="n">
         <v>187</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="45" t="n">
         <v>12</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="34">
         <f>C10*Supostos!$B$8+D10*Supostos!$B$5+E10*Supostos!$B$6+F10*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="34">
         <f>G10*12</f>
         <v/>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="35">
         <f>G10*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="35">
         <f>H10*Supostos!$B$9</f>
         <v/>
       </c>
@@ -1651,34 +1662,34 @@
           <t>Tarija</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
+      <c r="B11" s="45" t="n">
         <v>535000</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="32" t="n">
         <v>11</v>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D11" s="45" t="n">
         <v>264</v>
       </c>
-      <c r="E11" s="27" t="n">
+      <c r="E11" s="45" t="n">
         <v>17</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="34">
         <f>C11*Supostos!$B$8+D11*Supostos!$B$5+E11*Supostos!$B$6+F11*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="34">
         <f>G11*12</f>
         <v/>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="35">
         <f>G11*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="35">
         <f>H11*Supostos!$B$9</f>
         <v/>
       </c>
@@ -1694,34 +1705,34 @@
           <t>Beni</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
+      <c r="B12" s="45" t="n">
         <v>477000</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="32" t="n">
         <v>9</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="45" t="n">
         <v>222</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="45" t="n">
         <v>15</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="34">
         <f>C12*Supostos!$B$8+D12*Supostos!$B$5+E12*Supostos!$B$6+F12*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="34">
         <f>G12*12</f>
         <v/>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="35">
         <f>G12*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="35">
         <f>H12*Supostos!$B$9</f>
         <v/>
       </c>
@@ -1737,34 +1748,34 @@
           <t>Pando</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
+      <c r="B13" s="45" t="n">
         <v>131000</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="32" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="45" t="n">
         <v>70</v>
       </c>
-      <c r="E13" s="27" t="n">
+      <c r="E13" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="34">
         <f>C13*Supostos!$B$8+D13*Supostos!$B$5+E13*Supostos!$B$6+F13*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="34">
         <f>G13*12</f>
         <v/>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="35">
         <f>G13*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="35">
         <f>H13*Supostos!$B$9</f>
         <v/>
       </c>
@@ -1780,44 +1791,43 @@
           <t>BOLÍVIA (total)</t>
         </is>
       </c>
-      <c r="B14" s="28">
+      <c r="B14" s="46">
         <f>SUM(B5:B13)</f>
         <v/>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="46">
         <f>SUM(C5:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="28">
+      <c r="D14" s="46">
         <f>SUM(D5:D13)</f>
         <v/>
       </c>
-      <c r="E14" s="28">
+      <c r="E14" s="46">
         <f>SUM(E5:E13)</f>
         <v/>
       </c>
-      <c r="F14" s="28">
+      <c r="F14" s="46">
         <f>SUM(F5:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="37">
         <f>SUM(G5:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="37">
         <f>SUM(H5:H13)</f>
         <v/>
       </c>
-      <c r="I14" s="13">
+      <c r="I14" s="38">
         <f>SUM(I5:I13)</f>
         <v/>
       </c>
-      <c r="J14" s="13">
+      <c r="J14" s="38">
         <f>SUM(J5:J13)</f>
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
         <is>
@@ -1888,7 +1898,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1962,34 +1971,34 @@
           <t>Santa Cruz</t>
         </is>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="45" t="n">
         <v>1600000</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="32" t="n">
         <v>65</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="45" t="n">
         <v>10</v>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="45" t="n">
         <v>8</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="34">
         <f>D5*Supostos!$B$8+E5*Supostos!$B$5+F5*Supostos!$B$6+G5*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="34">
         <f>H5*12</f>
         <v/>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="35">
         <f>H5*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="35">
         <f>I5*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2010,34 +2019,34 @@
           <t>La Paz</t>
         </is>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="45" t="n">
         <v>760000</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="45" t="n">
         <v>150</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="45" t="n">
         <v>29</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="45" t="n">
         <v>17</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="34">
         <f>D6*Supostos!$B$8+E6*Supostos!$B$5+F6*Supostos!$B$6+G6*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="34">
         <f>H6*12</f>
         <v/>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="35">
         <f>H6*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K6" s="9">
+      <c r="K6" s="35">
         <f>I6*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2058,34 +2067,34 @@
           <t>La Paz</t>
         </is>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="45" t="n">
         <v>890000</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="45" t="n">
         <v>90</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="45" t="n">
         <v>6</v>
       </c>
-      <c r="G7" s="27" t="n">
+      <c r="G7" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="34">
         <f>D7*Supostos!$B$8+E7*Supostos!$B$5+F7*Supostos!$B$6+G7*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I7" s="8">
+      <c r="I7" s="34">
         <f>H7*12</f>
         <v/>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="35">
         <f>H7*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K7" s="9">
+      <c r="K7" s="35">
         <f>I7*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2106,34 +2115,34 @@
           <t>Cochabamba</t>
         </is>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="45" t="n">
         <v>670000</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="45" t="n">
         <v>60</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="45" t="n">
         <v>6</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="34">
         <f>D8*Supostos!$B$8+E8*Supostos!$B$5+F8*Supostos!$B$6+G8*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="34">
         <f>H8*12</f>
         <v/>
       </c>
-      <c r="J8" s="9">
+      <c r="J8" s="35">
         <f>H8*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="35">
         <f>I8*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2154,34 +2163,34 @@
           <t>Chuquisaca</t>
         </is>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="45" t="n">
         <v>300000</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="45" t="n">
         <v>30</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="34">
         <f>D9*Supostos!$B$8+E9*Supostos!$B$5+F9*Supostos!$B$6+G9*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I9" s="8">
+      <c r="I9" s="34">
         <f>H9*12</f>
         <v/>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="35">
         <f>H9*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="35">
         <f>I9*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2202,34 +2211,34 @@
           <t>Oruro</t>
         </is>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="45" t="n">
         <v>280000</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="45" t="n">
         <v>30</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="G10" s="27" t="n">
+      <c r="G10" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="34">
         <f>D10*Supostos!$B$8+E10*Supostos!$B$5+F10*Supostos!$B$6+G10*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="34">
         <f>H10*12</f>
         <v/>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="35">
         <f>H10*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="35">
         <f>I10*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2250,34 +2259,34 @@
           <t>Tarija</t>
         </is>
       </c>
-      <c r="C11" s="27" t="n">
+      <c r="C11" s="45" t="n">
         <v>270000</v>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D11" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="27" t="n">
+      <c r="E11" s="45" t="n">
         <v>30</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="27" t="n">
+      <c r="G11" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="34">
         <f>D11*Supostos!$B$8+E11*Supostos!$B$5+F11*Supostos!$B$6+G11*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="34">
         <f>H11*12</f>
         <v/>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="35">
         <f>H11*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K11" s="9">
+      <c r="K11" s="35">
         <f>I11*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2298,34 +2307,34 @@
           <t>Potosí</t>
         </is>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="45" t="n">
         <v>220000</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="45" t="n">
         <v>25</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="34">
         <f>D12*Supostos!$B$8+E12*Supostos!$B$5+F12*Supostos!$B$6+G12*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I12" s="8">
+      <c r="I12" s="34">
         <f>H12*12</f>
         <v/>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="35">
         <f>H12*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K12" s="9">
+      <c r="K12" s="35">
         <f>I12*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2346,34 +2355,34 @@
           <t>Cochabamba</t>
         </is>
       </c>
-      <c r="C13" s="27" t="n">
+      <c r="C13" s="45" t="n">
         <v>210000</v>
       </c>
-      <c r="D13" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="27" t="n">
+      <c r="D13" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="45" t="n">
         <v>20</v>
       </c>
-      <c r="F13" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="8">
+      <c r="F13" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="34">
         <f>D13*Supostos!$B$8+E13*Supostos!$B$5+F13*Supostos!$B$6+G13*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="34">
         <f>H13*12</f>
         <v/>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="35">
         <f>H13*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K13" s="9">
+      <c r="K13" s="35">
         <f>I13*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2394,34 +2403,34 @@
           <t>Cochabamba</t>
         </is>
       </c>
-      <c r="C14" s="27" t="n">
+      <c r="C14" s="45" t="n">
         <v>150000</v>
       </c>
-      <c r="D14" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="27" t="n">
+      <c r="D14" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="45" t="n">
         <v>15</v>
       </c>
-      <c r="F14" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="8">
+      <c r="F14" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="34">
         <f>D14*Supostos!$B$8+E14*Supostos!$B$5+F14*Supostos!$B$6+G14*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I14" s="8">
+      <c r="I14" s="34">
         <f>H14*12</f>
         <v/>
       </c>
-      <c r="J14" s="9">
+      <c r="J14" s="35">
         <f>H14*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K14" s="9">
+      <c r="K14" s="35">
         <f>I14*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2442,34 +2451,34 @@
           <t>Santa Cruz</t>
         </is>
       </c>
-      <c r="C15" s="27" t="n">
+      <c r="C15" s="45" t="n">
         <v>140000</v>
       </c>
-      <c r="D15" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="27" t="n">
+      <c r="D15" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="45" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="8">
+      <c r="G15" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="34">
         <f>D15*Supostos!$B$8+E15*Supostos!$B$5+F15*Supostos!$B$6+G15*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I15" s="8">
+      <c r="I15" s="34">
         <f>H15*12</f>
         <v/>
       </c>
-      <c r="J15" s="9">
+      <c r="J15" s="35">
         <f>H15*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K15" s="9">
+      <c r="K15" s="35">
         <f>I15*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2490,34 +2499,34 @@
           <t>Beni</t>
         </is>
       </c>
-      <c r="C16" s="27" t="n">
+      <c r="C16" s="45" t="n">
         <v>130000</v>
       </c>
-      <c r="D16" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="27" t="n">
+      <c r="D16" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="45" t="n">
         <v>15</v>
       </c>
-      <c r="F16" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="8">
+      <c r="F16" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="34">
         <f>D16*Supostos!$B$8+E16*Supostos!$B$5+F16*Supostos!$B$6+G16*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="34">
         <f>H16*12</f>
         <v/>
       </c>
-      <c r="J16" s="9">
+      <c r="J16" s="35">
         <f>H16*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K16" s="9">
+      <c r="K16" s="35">
         <f>I16*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2538,34 +2547,34 @@
           <t>Santa Cruz</t>
         </is>
       </c>
-      <c r="C17" s="27" t="n">
+      <c r="C17" s="45" t="n">
         <v>100000</v>
       </c>
-      <c r="D17" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="27" t="n">
+      <c r="D17" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="45" t="n">
         <v>10</v>
       </c>
-      <c r="F17" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8">
+      <c r="F17" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="34">
         <f>D17*Supostos!$B$8+E17*Supostos!$B$5+F17*Supostos!$B$6+G17*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="34">
         <f>H17*12</f>
         <v/>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="35">
         <f>H17*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="35">
         <f>I17*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2586,34 +2595,34 @@
           <t>Tarija</t>
         </is>
       </c>
-      <c r="C18" s="27" t="n">
+      <c r="C18" s="45" t="n">
         <v>100000</v>
       </c>
-      <c r="D18" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="27" t="n">
+      <c r="D18" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="45" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="8">
+      <c r="F18" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="34">
         <f>D18*Supostos!$B$8+E18*Supostos!$B$5+F18*Supostos!$B$6+G18*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I18" s="8">
+      <c r="I18" s="34">
         <f>H18*12</f>
         <v/>
       </c>
-      <c r="J18" s="9">
+      <c r="J18" s="35">
         <f>H18*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K18" s="9">
+      <c r="K18" s="35">
         <f>I18*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2634,34 +2643,34 @@
           <t>Beni</t>
         </is>
       </c>
-      <c r="C19" s="27" t="n">
+      <c r="C19" s="45" t="n">
         <v>100000</v>
       </c>
-      <c r="D19" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="27" t="n">
+      <c r="D19" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="45" t="n">
         <v>12</v>
       </c>
-      <c r="F19" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="8">
+      <c r="F19" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="34">
         <f>D19*Supostos!$B$8+E19*Supostos!$B$5+F19*Supostos!$B$6+G19*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I19" s="8">
+      <c r="I19" s="34">
         <f>H19*12</f>
         <v/>
       </c>
-      <c r="J19" s="9">
+      <c r="J19" s="35">
         <f>H19*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K19" s="9">
+      <c r="K19" s="35">
         <f>I19*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2682,34 +2691,34 @@
           <t>Pando</t>
         </is>
       </c>
-      <c r="C20" s="27" t="n">
+      <c r="C20" s="45" t="n">
         <v>70000</v>
       </c>
-      <c r="D20" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="27" t="n">
+      <c r="D20" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="45" t="n">
         <v>8</v>
       </c>
-      <c r="F20" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="8">
+      <c r="F20" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="45" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="34">
         <f>D20*Supostos!$B$8+E20*Supostos!$B$5+F20*Supostos!$B$6+G20*Supostos!$B$7</f>
         <v/>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="34">
         <f>H20*12</f>
         <v/>
       </c>
-      <c r="J20" s="9">
+      <c r="J20" s="35">
         <f>H20*Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K20" s="9">
+      <c r="K20" s="35">
         <f>I20*Supostos!$B$9</f>
         <v/>
       </c>
@@ -2725,39 +2734,39 @@
           <t>Total das 16 cidades</t>
         </is>
       </c>
-      <c r="C21" s="28">
+      <c r="C21" s="46">
         <f>SUM(C5:C20)</f>
         <v/>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="46">
         <f>SUM(D5:D20)</f>
         <v/>
       </c>
-      <c r="E21" s="28">
+      <c r="E21" s="46">
         <f>SUM(E5:E20)</f>
         <v/>
       </c>
-      <c r="F21" s="28">
+      <c r="F21" s="46">
         <f>SUM(F5:F20)</f>
         <v/>
       </c>
-      <c r="G21" s="28">
+      <c r="G21" s="46">
         <f>SUM(G5:G20)</f>
         <v/>
       </c>
-      <c r="H21" s="12">
+      <c r="H21" s="37">
         <f>SUM(H5:H20)</f>
         <v/>
       </c>
-      <c r="I21" s="12">
+      <c r="I21" s="37">
         <f>SUM(I5:I20)</f>
         <v/>
       </c>
-      <c r="J21" s="13">
+      <c r="J21" s="38">
         <f>SUM(J5:J20)</f>
         <v/>
       </c>
-      <c r="K21" s="13">
+      <c r="K21" s="38">
         <f>SUM(K5:K20)</f>
         <v/>
       </c>
@@ -2768,12 +2777,11 @@
           <t>Participação das 16 cidades na receita da Bolívia</t>
         </is>
       </c>
-      <c r="I22" s="30">
+      <c r="I22" s="47">
         <f>IFERROR(I21/Departamentos!H14,0)</f>
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
@@ -2823,7 +2831,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2897,7 +2904,7 @@
           <t>Você: visão, vendas grandes, relação com Ministério e SEDES, decisão clínica do produto.</t>
         </is>
       </c>
-      <c r="C5" s="31" t="n">
+      <c r="C5" s="48" t="n">
         <v>12000</v>
       </c>
       <c r="D5" s="24" t="n">
@@ -2915,19 +2922,19 @@
       <c r="H5" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="35">
         <f>$C5*E5*(1+IF($D5=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="35">
         <f>$C5*F5*(1+IF($D5=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="35">
         <f>$C5*G5*(1+IF($D5=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="35">
         <f>$C5*H5*(1+IF($D5=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -2943,7 +2950,7 @@
           <t>Arquitetura, segurança, revisão de código, banco de dados e desempenho.</t>
         </is>
       </c>
-      <c r="C6" s="31" t="n">
+      <c r="C6" s="48" t="n">
         <v>15000</v>
       </c>
       <c r="D6" s="24" t="n">
@@ -2961,19 +2968,19 @@
       <c r="H6" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="35">
         <f>$C6*E6*(1+IF($D6=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="35">
         <f>$C6*F6*(1+IF($D6=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K6" s="9">
+      <c r="K6" s="35">
         <f>$C6*G6*(1+IF($D6=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L6" s="9">
+      <c r="L6" s="35">
         <f>$C6*H6*(1+IF($D6=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -2989,7 +2996,7 @@
           <t>Programa módulos novos e correções.</t>
         </is>
       </c>
-      <c r="C7" s="31" t="n">
+      <c r="C7" s="48" t="n">
         <v>9000</v>
       </c>
       <c r="D7" s="24" t="n">
@@ -3007,19 +3014,19 @@
       <c r="H7" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="35">
         <f>$C7*E7*(1+IF($D7=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="35">
         <f>$C7*F7*(1+IF($D7=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K7" s="9">
+      <c r="K7" s="35">
         <f>$C7*G7*(1+IF($D7=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L7" s="9">
+      <c r="L7" s="35">
         <f>$C7*H7*(1+IF($D7=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3035,7 +3042,7 @@
           <t>Ajustes, relatórios, telas simples, testes.</t>
         </is>
       </c>
-      <c r="C8" s="31" t="n">
+      <c r="C8" s="48" t="n">
         <v>5000</v>
       </c>
       <c r="D8" s="24" t="n">
@@ -3053,19 +3060,19 @@
       <c r="H8" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="35">
         <f>$C8*E8*(1+IF($D8=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J8" s="9">
+      <c r="J8" s="35">
         <f>$C8*F8*(1+IF($D8=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="35">
         <f>$C8*G8*(1+IF($D8=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="35">
         <f>$C8*H8*(1+IF($D8=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3081,7 +3088,7 @@
           <t>Servidores, backups, monitoramento, cópias de segurança, auditoria de acesso.</t>
         </is>
       </c>
-      <c r="C9" s="31" t="n">
+      <c r="C9" s="48" t="n">
         <v>12000</v>
       </c>
       <c r="D9" s="24" t="n">
@@ -3099,19 +3106,19 @@
       <c r="H9" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="35">
         <f>$C9*E9*(1+IF($D9=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="35">
         <f>$C9*F9*(1+IF($D9=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="35">
         <f>$C9*G9*(1+IF($D9=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="35">
         <f>$C9*H9*(1+IF($D9=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3127,7 +3134,7 @@
           <t>Testa cada versão antes de chegar aos centros.</t>
         </is>
       </c>
-      <c r="C10" s="31" t="n">
+      <c r="C10" s="48" t="n">
         <v>6000</v>
       </c>
       <c r="D10" s="24" t="n">
@@ -3145,19 +3152,19 @@
       <c r="H10" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="35">
         <f>$C10*E10*(1+IF($D10=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="35">
         <f>$C10*F10*(1+IF($D10=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="35">
         <f>$C10*G10*(1+IF($D10=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L10" s="9">
+      <c r="L10" s="35">
         <f>$C10*H10*(1+IF($D10=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3173,7 +3180,7 @@
           <t>Atende telefone e WhatsApp dos centros; ~1 pessoa a cada 300 estabelecimentos.</t>
         </is>
       </c>
-      <c r="C11" s="31" t="n">
+      <c r="C11" s="48" t="n">
         <v>4000</v>
       </c>
       <c r="D11" s="24" t="n">
@@ -3191,19 +3198,19 @@
       <c r="H11" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="35">
         <f>$C11*E11*(1+IF($D11=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="35">
         <f>$C11*F11*(1+IF($D11=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K11" s="9">
+      <c r="K11" s="35">
         <f>$C11*G11*(1+IF($D11=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L11" s="9">
+      <c r="L11" s="35">
         <f>$C11*H11*(1+IF($D11=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3219,7 +3226,7 @@
           <t>Resolve o que o nível 1 não resolve; acesso ao banco.</t>
         </is>
       </c>
-      <c r="C12" s="31" t="n">
+      <c r="C12" s="48" t="n">
         <v>6500</v>
       </c>
       <c r="D12" s="24" t="n">
@@ -3237,19 +3244,19 @@
       <c r="H12" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="35">
         <f>$C12*E12*(1+IF($D12=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="35">
         <f>$C12*F12*(1+IF($D12=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K12" s="9">
+      <c r="K12" s="35">
         <f>$C12*G12*(1+IF($D12=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L12" s="9">
+      <c r="L12" s="35">
         <f>$C12*H12*(1+IF($D12=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3265,7 +3272,7 @@
           <t>Vai aos centros, cadastra usuários, capacita o pessoal.</t>
         </is>
       </c>
-      <c r="C13" s="31" t="n">
+      <c r="C13" s="48" t="n">
         <v>6000</v>
       </c>
       <c r="D13" s="24" t="n">
@@ -3283,19 +3290,19 @@
       <c r="H13" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="35">
         <f>$C13*E13*(1+IF($D13=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="35">
         <f>$C13*F13*(1+IF($D13=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K13" s="9">
+      <c r="K13" s="35">
         <f>$C13*G13*(1+IF($D13=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L13" s="9">
+      <c r="L13" s="35">
         <f>$C13*H13*(1+IF($D13=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3311,7 +3318,7 @@
           <t>Responde por uma região (vários departamentos): implantação, SEDES e redes.</t>
         </is>
       </c>
-      <c r="C14" s="31" t="n">
+      <c r="C14" s="48" t="n">
         <v>9000</v>
       </c>
       <c r="D14" s="24" t="n">
@@ -3329,19 +3336,19 @@
       <c r="H14" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="35">
         <f>$C14*E14*(1+IF($D14=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J14" s="9">
+      <c r="J14" s="35">
         <f>$C14*F14*(1+IF($D14=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K14" s="9">
+      <c r="K14" s="35">
         <f>$C14*G14*(1+IF($D14=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L14" s="9">
+      <c r="L14" s="35">
         <f>$C14*H14*(1+IF($D14=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3357,7 +3364,7 @@
           <t>Valida fluxos clínicos, formulários oficiais e normas do Ministério.</t>
         </is>
       </c>
-      <c r="C15" s="31" t="n">
+      <c r="C15" s="48" t="n">
         <v>10000</v>
       </c>
       <c r="D15" s="24" t="n">
@@ -3375,19 +3382,19 @@
       <c r="H15" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="I15" s="9">
+      <c r="I15" s="35">
         <f>$C15*E15*(1+IF($D15=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J15" s="9">
+      <c r="J15" s="35">
         <f>$C15*F15*(1+IF($D15=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K15" s="9">
+      <c r="K15" s="35">
         <f>$C15*G15*(1+IF($D15=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L15" s="9">
+      <c r="L15" s="35">
         <f>$C15*H15*(1+IF($D15=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3403,7 +3410,7 @@
           <t>Licitações, SICOES, propostas, contratos com municípios e governações.</t>
         </is>
       </c>
-      <c r="C16" s="31" t="n">
+      <c r="C16" s="48" t="n">
         <v>10000</v>
       </c>
       <c r="D16" s="24" t="n">
@@ -3421,19 +3428,19 @@
       <c r="H16" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="35">
         <f>$C16*E16*(1+IF($D16=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J16" s="9">
+      <c r="J16" s="35">
         <f>$C16*F16*(1+IF($D16=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K16" s="9">
+      <c r="K16" s="35">
         <f>$C16*G16*(1+IF($D16=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L16" s="9">
+      <c r="L16" s="35">
         <f>$C16*H16*(1+IF($D16=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3449,7 +3456,7 @@
           <t>Cronogramas de implantação, indicadores de atendimento, equipe de campo.</t>
         </is>
       </c>
-      <c r="C17" s="31" t="n">
+      <c r="C17" s="48" t="n">
         <v>11000</v>
       </c>
       <c r="D17" s="24" t="n">
@@ -3467,19 +3474,19 @@
       <c r="H17" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="35">
         <f>$C17*E17*(1+IF($D17=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="35">
         <f>$C17*F17*(1+IF($D17=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="35">
         <f>$C17*G17*(1+IF($D17=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L17" s="9">
+      <c r="L17" s="35">
         <f>$C17*H17*(1+IF($D17=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3495,7 +3502,7 @@
           <t>Telas, capacitação visual, materiais.</t>
         </is>
       </c>
-      <c r="C18" s="31" t="n">
+      <c r="C18" s="48" t="n">
         <v>6000</v>
       </c>
       <c r="D18" s="24" t="n">
@@ -3513,19 +3520,19 @@
       <c r="H18" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="9">
+      <c r="I18" s="35">
         <f>$C18*E18*(1+IF($D18=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J18" s="9">
+      <c r="J18" s="35">
         <f>$C18*F18*(1+IF($D18=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K18" s="9">
+      <c r="K18" s="35">
         <f>$C18*G18*(1+IF($D18=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L18" s="9">
+      <c r="L18" s="35">
         <f>$C18*H18*(1+IF($D18=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3541,7 +3548,7 @@
           <t>Faturas, cobranças, pagamentos, folha.</t>
         </is>
       </c>
-      <c r="C19" s="31" t="n">
+      <c r="C19" s="48" t="n">
         <v>5000</v>
       </c>
       <c r="D19" s="24" t="n">
@@ -3559,19 +3566,19 @@
       <c r="H19" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="I19" s="9">
+      <c r="I19" s="35">
         <f>$C19*E19*(1+IF($D19=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J19" s="9">
+      <c r="J19" s="35">
         <f>$C19*F19*(1+IF($D19=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K19" s="9">
+      <c r="K19" s="35">
         <f>$C19*G19*(1+IF($D19=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L19" s="9">
+      <c r="L19" s="35">
         <f>$C19*H19*(1+IF($D19=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3587,7 +3594,7 @@
           <t>Impostos, balanços, folha.</t>
         </is>
       </c>
-      <c r="C20" s="31" t="n">
+      <c r="C20" s="48" t="n">
         <v>2500</v>
       </c>
       <c r="D20" s="24" t="n">
@@ -3605,19 +3612,19 @@
       <c r="H20" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="9">
+      <c r="I20" s="35">
         <f>$C20*E20*(1+IF($D20=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J20" s="9">
+      <c r="J20" s="35">
         <f>$C20*F20*(1+IF($D20=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K20" s="9">
+      <c r="K20" s="35">
         <f>$C20*G20*(1+IF($D20=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L20" s="9">
+      <c r="L20" s="35">
         <f>$C20*H20*(1+IF($D20=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3633,7 +3640,7 @@
           <t>Contratos, SENAPI, proteção de dados, licitações.</t>
         </is>
       </c>
-      <c r="C21" s="31" t="n">
+      <c r="C21" s="48" t="n">
         <v>3000</v>
       </c>
       <c r="D21" s="24" t="n">
@@ -3651,19 +3658,19 @@
       <c r="H21" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="9">
+      <c r="I21" s="35">
         <f>$C21*E21*(1+IF($D21=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="J21" s="9">
+      <c r="J21" s="35">
         <f>$C21*F21*(1+IF($D21=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="K21" s="9">
+      <c r="K21" s="35">
         <f>$C21*G21*(1+IF($D21=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
-      <c r="L21" s="9">
+      <c r="L21" s="35">
         <f>$C21*H21*(1+IF($D21=1,0,Supostos!$B$12))</f>
         <v/>
       </c>
@@ -3674,35 +3681,35 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E22" s="28">
+      <c r="E22" s="46">
         <f>SUM(E5:E21)</f>
         <v/>
       </c>
-      <c r="F22" s="28">
+      <c r="F22" s="46">
         <f>SUM(F5:F21)</f>
         <v/>
       </c>
-      <c r="G22" s="28">
+      <c r="G22" s="46">
         <f>SUM(G5:G21)</f>
         <v/>
       </c>
-      <c r="H22" s="28">
+      <c r="H22" s="46">
         <f>SUM(H5:H21)</f>
         <v/>
       </c>
-      <c r="I22" s="13">
+      <c r="I22" s="38">
         <f>SUM(I5:I21)</f>
         <v/>
       </c>
-      <c r="J22" s="13">
+      <c r="J22" s="38">
         <f>SUM(J5:J21)</f>
         <v/>
       </c>
-      <c r="K22" s="13">
+      <c r="K22" s="38">
         <f>SUM(K5:K21)</f>
         <v/>
       </c>
-      <c r="L22" s="13">
+      <c r="L22" s="38">
         <f>SUM(L5:L21)</f>
         <v/>
       </c>
@@ -3713,24 +3720,23 @@
           <t>Custo mensal da equipe (US$)</t>
         </is>
       </c>
-      <c r="I23" s="8">
+      <c r="I23" s="34">
         <f>I22/Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="J23" s="8">
+      <c r="J23" s="34">
         <f>J22/Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="K23" s="8">
+      <c r="K23" s="34">
         <f>K22/Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="L23" s="8">
+      <c r="L23" s="34">
         <f>L22/Supostos!$B$9</f>
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
         <is>
@@ -3776,7 +3782,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3840,16 +3845,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="41" t="n">
         <v>40</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="41" t="n">
         <v>135</v>
       </c>
-      <c r="G5" s="18" t="n">
+      <c r="G5" s="41" t="n">
         <v>809</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="41" t="n">
         <v>2519</v>
       </c>
     </row>
@@ -3874,16 +3879,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E6" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="18" t="n">
+      <c r="E6" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="41" t="n">
         <v>20</v>
       </c>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="41" t="n">
         <v>20</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H6" s="41" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3908,16 +3913,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="41" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3942,16 +3947,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E8" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="18" t="n">
+      <c r="E8" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="41" t="n">
         <v>20</v>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="41" t="n">
         <v>200</v>
       </c>
     </row>
@@ -3976,16 +3981,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="41" t="n">
         <v>30</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="41" t="n">
         <v>150</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G9" s="41" t="n">
         <v>500</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="41" t="n">
         <v>3000</v>
       </c>
     </row>
@@ -4010,16 +4015,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E10" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="18" t="n">
+      <c r="E10" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="41" t="n">
         <v>26</v>
       </c>
-      <c r="G10" s="18" t="n">
+      <c r="G10" s="41" t="n">
         <v>80</v>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="41" t="n">
         <v>300</v>
       </c>
     </row>
@@ -4044,16 +4049,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E11" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="18" t="n">
+      <c r="E11" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="41" t="n">
         <v>25</v>
       </c>
-      <c r="G11" s="18" t="n">
+      <c r="G11" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="H11" s="18" t="n">
+      <c r="H11" s="41" t="n">
         <v>100</v>
       </c>
     </row>
@@ -4078,16 +4083,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="41" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="41" t="n">
         <v>20</v>
       </c>
-      <c r="G12" s="18" t="n">
+      <c r="G12" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="H12" s="18" t="n">
+      <c r="H12" s="41" t="n">
         <v>200</v>
       </c>
     </row>
@@ -4112,16 +4117,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="18" t="n">
+      <c r="E13" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="G13" s="41" t="n">
         <v>800</v>
       </c>
-      <c r="H13" s="18" t="n">
+      <c r="H13" s="41" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -4146,16 +4151,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E14" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="18" t="n">
+      <c r="E14" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="41" t="n">
         <v>100</v>
       </c>
-      <c r="G14" s="18" t="n">
+      <c r="G14" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="H14" s="18" t="n">
+      <c r="H14" s="41" t="n">
         <v>500</v>
       </c>
     </row>
@@ -4180,16 +4185,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E15" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="18" t="n">
+      <c r="E15" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="G15" s="18" t="n">
+      <c r="G15" s="41" t="n">
         <v>1500</v>
       </c>
-      <c r="H15" s="18" t="n">
+      <c r="H15" s="41" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -4214,16 +4219,16 @@
           <t>fixo</t>
         </is>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="G16" s="18" t="n">
+      <c r="G16" s="41" t="n">
         <v>800</v>
       </c>
-      <c r="H16" s="18" t="n">
+      <c r="H16" s="41" t="n">
         <v>3000</v>
       </c>
     </row>
@@ -4248,19 +4253,19 @@
           <t>por pessoa</t>
         </is>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="36">
         <f>7*Equipe!E22</f>
         <v/>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="36">
         <f>7*Equipe!F22</f>
         <v/>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="36">
         <f>7*Equipe!G22</f>
         <v/>
       </c>
-      <c r="H17" s="10">
+      <c r="H17" s="36">
         <f>7*Equipe!H22</f>
         <v/>
       </c>
@@ -4286,19 +4291,19 @@
           <t>por pessoa</t>
         </is>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="36">
         <f>15*Equipe!E22</f>
         <v/>
       </c>
-      <c r="F18" s="10">
+      <c r="F18" s="36">
         <f>15*Equipe!F22</f>
         <v/>
       </c>
-      <c r="G18" s="10">
+      <c r="G18" s="36">
         <f>15*Equipe!G22</f>
         <v/>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="36">
         <f>15*Equipe!H22</f>
         <v/>
       </c>
@@ -4324,19 +4329,19 @@
           <t>por pessoa</t>
         </is>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="36">
         <f>4*Equipe!E22</f>
         <v/>
       </c>
-      <c r="F19" s="10">
+      <c r="F19" s="36">
         <f>4*Equipe!F22</f>
         <v/>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="36">
         <f>4*Equipe!G22</f>
         <v/>
       </c>
-      <c r="H19" s="10">
+      <c r="H19" s="36">
         <f>4*Equipe!H22</f>
         <v/>
       </c>
@@ -4362,19 +4367,19 @@
           <t>por pessoa</t>
         </is>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="36">
         <f>4*Equipe!E22</f>
         <v/>
       </c>
-      <c r="F20" s="10">
+      <c r="F20" s="36">
         <f>4*Equipe!F22</f>
         <v/>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="36">
         <f>4*Equipe!G22</f>
         <v/>
       </c>
-      <c r="H20" s="10">
+      <c r="H20" s="36">
         <f>4*Equipe!H22</f>
         <v/>
       </c>
@@ -4400,19 +4405,19 @@
           <t>por pessoa</t>
         </is>
       </c>
-      <c r="E21" s="10">
+      <c r="E21" s="36">
         <f>28*Equipe!E22</f>
         <v/>
       </c>
-      <c r="F21" s="10">
+      <c r="F21" s="36">
         <f>28*Equipe!F22</f>
         <v/>
       </c>
-      <c r="G21" s="10">
+      <c r="G21" s="36">
         <f>28*Equipe!G22</f>
         <v/>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="36">
         <f>28*Equipe!H22</f>
         <v/>
       </c>
@@ -4423,24 +4428,23 @@
           <t>TOTAL ferramentas (US$/mês)</t>
         </is>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="37">
         <f>SUM(E5:E21)</f>
         <v/>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="37">
         <f>SUM(F5:F21)</f>
         <v/>
       </c>
-      <c r="G22" s="12">
+      <c r="G22" s="37">
         <f>SUM(G5:G21)</f>
         <v/>
       </c>
-      <c r="H22" s="12">
+      <c r="H22" s="37">
         <f>SUM(H5:H21)</f>
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>

</xml_diff>